<commit_message>
Deploy verified dashboard and input fixes
</commit_message>
<xml_diff>
--- a/Testing User Guide.xlsx
+++ b/Testing User Guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\New-rafiqi-central-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF0DD52F-1350-4770-B850-C856666AD735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB5C8B2-1F70-43D1-ACA5-70D52C0BEE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{46839000-F319-4EEB-9279-DCF91A1AE02A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t xml:space="preserve">Mode </t>
   </si>
@@ -93,7 +93,7 @@
     <t>Nia Margin</t>
   </si>
   <si>
-    <t xml:space="preserve">User Input ( TEAM_FINANCE_DAILY ) - Most CM2 Fill hona jarui he in this tab </t>
+    <t xml:space="preserve">User Input ( TEAM_FINANCE_DAILY / TEAM_REQ_POLICY_REGISTRY / TEAM_REQ_ACTION_LOG / TEAM_REQ_EVIDENCE_LOG ) - Most CM2 Fill hona jarui he in this tab and inme Owenr koi aur rahega and approver + verifier koi aur rahega  </t>
   </si>
 </sst>
 </file>
@@ -559,7 +559,10 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>1</v>
+      </c>
       <c r="B6" s="2" t="s">
         <v>18</v>
       </c>

</xml_diff>

<commit_message>
Adopt final RafiQi UI and reconnect live dashboard data
</commit_message>
<xml_diff>
--- a/Testing User Guide.xlsx
+++ b/Testing User Guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\New-rafiqi-central-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB5C8B2-1F70-43D1-ACA5-70D52C0BEE2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84622F5B-31FC-4AF9-96D1-7291B41BED38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{46839000-F319-4EEB-9279-DCF91A1AE02A}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t xml:space="preserve">Mode </t>
   </si>
@@ -94,6 +94,12 @@
   </si>
   <si>
     <t xml:space="preserve">User Input ( TEAM_FINANCE_DAILY / TEAM_REQ_POLICY_REGISTRY / TEAM_REQ_ACTION_LOG / TEAM_REQ_EVIDENCE_LOG ) - Most CM2 Fill hona jarui he in this tab and inme Owenr koi aur rahega and approver + verifier koi aur rahega  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nia Growth </t>
+  </si>
+  <si>
+    <t>User input ( TEAM_NIA_GROWTH )</t>
   </si>
 </sst>
 </file>
@@ -474,7 +480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A8782B9-1AEC-4658-9C24-2FF4BCD5C0F7}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
@@ -570,6 +576,17 @@
         <v>19</v>
       </c>
     </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>